<commit_message>
fix: Nigeria 1200→1330 NGN gas, 1250→1600 NGN diesel (NNPC March 2026)
</commit_message>
<xml_diff>
--- a/africa_fuel_tracker_latest.xlsx
+++ b/africa_fuel_tracker_latest.xlsx
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>$1.168</t>
+          <t>$1.169</t>
         </is>
       </c>
       <c r="D6" s="12" t="inlineStr">
@@ -1673,12 +1673,12 @@
       </c>
       <c r="F6" s="14" t="inlineStr">
         <is>
-          <t>+39.1%</t>
+          <t>+40.0%</t>
         </is>
       </c>
       <c r="G6" s="15" t="inlineStr">
         <is>
-          <t>$1.131</t>
+          <t>$1.135</t>
         </is>
       </c>
     </row>
@@ -1705,7 +1705,7 @@
       </c>
       <c r="F7" s="20" t="inlineStr">
         <is>
-          <t>Somalia</t>
+          <t>Nigeria</t>
         </is>
       </c>
       <c r="G7" s="21" t="inlineStr">
@@ -1787,10 +1787,10 @@
         <v>16</v>
       </c>
       <c r="D13" s="31" t="n">
-        <v>1.13806875</v>
+        <v>1.14308125</v>
       </c>
       <c r="E13" s="31" t="n">
-        <v>1.12975</v>
+        <v>1.14324375</v>
       </c>
       <c r="F13" s="32" t="n">
         <v>0.6522</v>
@@ -2914,23 +2914,23 @@
         </is>
       </c>
       <c r="E23" s="66" t="n">
-        <v>0.7403</v>
+        <v>0.8205</v>
       </c>
       <c r="F23" s="66" t="n">
-        <v>0.7711</v>
+        <v>0.987</v>
       </c>
       <c r="G23" s="67" t="n">
-        <v>1200</v>
+        <v>1330</v>
       </c>
       <c r="H23" s="67" t="n">
-        <v>1250</v>
+        <v>1600</v>
       </c>
       <c r="I23" s="68" t="n">
         <v>1621</v>
       </c>
       <c r="J23" s="72" t="inlineStr">
         <is>
-          <t>▲ +26.3%</t>
+          <t>▲ +40.0%</t>
         </is>
       </c>
       <c r="K23" s="69" t="inlineStr">
@@ -4612,10 +4612,10 @@
         </is>
       </c>
       <c r="E63" s="77" t="n">
-        <v>1.167846296296296</v>
+        <v>1.169331481481481</v>
       </c>
       <c r="F63" s="77" t="n">
-        <v>1.131401851851852</v>
+        <v>1.1354</v>
       </c>
       <c r="G63" s="78" t="n"/>
       <c r="H63" s="78" t="n"/>
@@ -5613,29 +5613,29 @@
         <v>0.5861</v>
       </c>
       <c r="D24" s="91" t="n">
-        <v>0.7403</v>
+        <v>0.8205</v>
       </c>
       <c r="E24" s="72" t="inlineStr">
         <is>
-          <t>▲ +26.3%</t>
+          <t>▲ +40.0%</t>
         </is>
       </c>
       <c r="F24" s="90" t="n">
         <v>0.7403</v>
       </c>
       <c r="G24" s="91" t="n">
-        <v>0.7711</v>
+        <v>0.987</v>
       </c>
       <c r="H24" s="72" t="inlineStr">
         <is>
-          <t>▲ +4.2%</t>
+          <t>▲ +33.3%</t>
         </is>
       </c>
       <c r="I24" s="58" t="n">
-        <v>1200</v>
+        <v>1330</v>
       </c>
       <c r="J24" s="58" t="n">
-        <v>1250</v>
+        <v>1600</v>
       </c>
       <c r="K24" s="61" t="inlineStr">
         <is>
@@ -7650,23 +7650,23 @@
       </c>
       <c r="G11" s="113" t="inlineStr">
         <is>
-          <t xml:space="preserve">  7.  Nigeria</t>
+          <t xml:space="preserve">  7.  Botswana</t>
         </is>
       </c>
       <c r="H11" s="100" t="inlineStr">
         <is>
-          <t>West Africa</t>
+          <t>Southern Africa</t>
         </is>
       </c>
       <c r="I11" s="101" t="n">
-        <v>0.7403</v>
+        <v>0.7792</v>
       </c>
       <c r="J11" s="102" t="n">
-        <v>0.7711</v>
-      </c>
-      <c r="K11" s="114" t="inlineStr">
-        <is>
-          <t>▲ +26.3%</t>
+        <v>0.7792</v>
+      </c>
+      <c r="K11" s="112" t="inlineStr">
+        <is>
+          <t>▼ -31.8%</t>
         </is>
       </c>
     </row>
@@ -7694,23 +7694,23 @@
       </c>
       <c r="G12" s="110" t="inlineStr">
         <is>
-          <t xml:space="preserve">  8.  Botswana</t>
+          <t xml:space="preserve">  8.  Nigeria</t>
         </is>
       </c>
       <c r="H12" s="106" t="inlineStr">
         <is>
-          <t>Southern Africa</t>
+          <t>West Africa</t>
         </is>
       </c>
       <c r="I12" s="107" t="n">
-        <v>0.7792</v>
+        <v>0.8205</v>
       </c>
       <c r="J12" s="108" t="n">
-        <v>0.7792</v>
-      </c>
-      <c r="K12" s="112" t="inlineStr">
-        <is>
-          <t>▼ -31.8%</t>
+        <v>0.987</v>
+      </c>
+      <c r="K12" s="114" t="inlineStr">
+        <is>
+          <t>▲ +40.0%</t>
         </is>
       </c>
     </row>
@@ -7850,38 +7850,38 @@
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="53" t="inlineStr">
         <is>
-          <t>Somalia</t>
+          <t>Nigeria</t>
         </is>
       </c>
       <c r="B19" s="54" t="inlineStr">
         <is>
-          <t>East Africa</t>
+          <t>West Africa</t>
         </is>
       </c>
       <c r="C19" s="116" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>NGN</t>
         </is>
       </c>
       <c r="D19" s="88" t="n">
-        <v>1.15</v>
+        <v>0.5861</v>
       </c>
       <c r="E19" s="91" t="n">
-        <v>1.6</v>
+        <v>0.8205</v>
       </c>
       <c r="F19" s="72" t="inlineStr">
         <is>
-          <t>▲ +39.1%</t>
+          <t>▲ +40.0%</t>
         </is>
       </c>
       <c r="G19" s="117" t="n">
-        <v>0.45</v>
+        <v>0.2344</v>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="62" t="inlineStr">
         <is>
-          <t>Ethiopia</t>
+          <t>Somalia</t>
         </is>
       </c>
       <c r="B20" s="63" t="inlineStr">
@@ -7891,53 +7891,53 @@
       </c>
       <c r="C20" s="118" t="inlineStr">
         <is>
-          <t>ETB</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="D20" s="88" t="n">
-        <v>0.6447000000000001</v>
+        <v>1.15</v>
       </c>
       <c r="E20" s="89" t="n">
-        <v>0.8398</v>
+        <v>1.6</v>
       </c>
       <c r="F20" s="72" t="inlineStr">
         <is>
-          <t>▲ +30.3%</t>
+          <t>▲ +39.1%</t>
         </is>
       </c>
       <c r="G20" s="117" t="n">
-        <v>0.1951</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="53" t="inlineStr">
         <is>
-          <t>Nigeria</t>
+          <t>Ethiopia</t>
         </is>
       </c>
       <c r="B21" s="54" t="inlineStr">
         <is>
-          <t>West Africa</t>
+          <t>East Africa</t>
         </is>
       </c>
       <c r="C21" s="116" t="inlineStr">
         <is>
-          <t>NGN</t>
+          <t>ETB</t>
         </is>
       </c>
       <c r="D21" s="88" t="n">
-        <v>0.5861</v>
+        <v>0.6447000000000001</v>
       </c>
       <c r="E21" s="91" t="n">
-        <v>0.7403</v>
+        <v>0.8398</v>
       </c>
       <c r="F21" s="72" t="inlineStr">
         <is>
-          <t>▲ +26.3%</t>
+          <t>▲ +30.3%</t>
         </is>
       </c>
       <c r="G21" s="117" t="n">
-        <v>0.1542</v>
+        <v>0.1951</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
@@ -9045,10 +9045,10 @@
       </c>
       <c r="B14" s="129" t="n"/>
       <c r="C14" s="130" t="n">
-        <v>1.13806875</v>
+        <v>1.14308125</v>
       </c>
       <c r="D14" s="130" t="n">
-        <v>1.12975</v>
+        <v>1.14324375</v>
       </c>
       <c r="E14" s="131" t="n">
         <v>0.6522</v>
@@ -9521,20 +9521,20 @@
         </is>
       </c>
       <c r="C28" s="57" t="n">
-        <v>0.7403</v>
+        <v>0.8205</v>
       </c>
       <c r="D28" s="57" t="n">
-        <v>0.7711</v>
+        <v>0.987</v>
       </c>
       <c r="E28" s="58" t="n">
-        <v>1200</v>
+        <v>1330</v>
       </c>
       <c r="F28" s="58" t="n">
-        <v>1250</v>
+        <v>1600</v>
       </c>
       <c r="G28" s="72" t="inlineStr">
         <is>
-          <t>▲ +26.3%</t>
+          <t>▲ +40.0%</t>
         </is>
       </c>
       <c r="H28" s="61" t="inlineStr">

</xml_diff>

<commit_message>
chore: regenerate dashboard + Excel 2026-03-31
</commit_message>
<xml_diff>
--- a/africa_fuel_tracker_latest.xlsx
+++ b/africa_fuel_tracker_latest.xlsx
@@ -1768,7 +1768,7 @@
         <v>0.6327166666666667</v>
       </c>
       <c r="E12" s="26" t="n">
-        <v>0.60015</v>
+        <v>0.6001500000000001</v>
       </c>
       <c r="F12" s="27" t="n">
         <v>0.0309</v>
@@ -8772,7 +8772,7 @@
         <v>0.6327166666666667</v>
       </c>
       <c r="D4" s="123" t="n">
-        <v>0.60015</v>
+        <v>0.6001500000000001</v>
       </c>
       <c r="E4" s="124" t="n">
         <v>0.0309</v>

</xml_diff>